<commit_message>
Otomatik veri güncelleme (24.07.2026 13:07 UTC)
</commit_message>
<xml_diff>
--- a/kredi mevduat/kredi_mevduat.xlsx
+++ b/kredi mevduat/kredi_mevduat.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H603"/>
+  <dimension ref="A1:H604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16116,6 +16116,32 @@
       </c>
       <c r="H603" t="n">
         <v>8.220000000000001</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B604" t="n">
+        <v>64.98</v>
+      </c>
+      <c r="C604" t="n">
+        <v>47.26</v>
+      </c>
+      <c r="D604" t="n">
+        <v>41.23</v>
+      </c>
+      <c r="E604" t="n">
+        <v>53.75</v>
+      </c>
+      <c r="F604" t="n">
+        <v>63.41</v>
+      </c>
+      <c r="G604" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="H604" t="n">
+        <v>7.95</v>
       </c>
     </row>
   </sheetData>
@@ -16129,7 +16155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K603"/>
+  <dimension ref="A1:K604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37257,6 +37283,41 @@
       </c>
       <c r="K603" t="n">
         <v>2.13</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B604" t="n">
+        <v>46.13</v>
+      </c>
+      <c r="C604" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="D604" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="E604" t="n">
+        <v>43.26</v>
+      </c>
+      <c r="F604" t="n">
+        <v>39.35</v>
+      </c>
+      <c r="G604" t="n">
+        <v>46.72</v>
+      </c>
+      <c r="H604" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="I604" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="J604" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="K604" t="n">
+        <v>2.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Otomatik veri güncelleme (31.07.2026 13:21 UTC)
</commit_message>
<xml_diff>
--- a/kredi mevduat/kredi_mevduat.xlsx
+++ b/kredi mevduat/kredi_mevduat.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H604"/>
+  <dimension ref="A1:H605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16142,6 +16142,32 @@
       </c>
       <c r="H604" t="n">
         <v>7.95</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B605" t="n">
+        <v>65.16</v>
+      </c>
+      <c r="C605" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="D605" t="n">
+        <v>41.39</v>
+      </c>
+      <c r="E605" t="n">
+        <v>54.39</v>
+      </c>
+      <c r="F605" t="n">
+        <v>63.47</v>
+      </c>
+      <c r="G605" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="H605" t="n">
+        <v>7.92</v>
       </c>
     </row>
   </sheetData>
@@ -16155,7 +16181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K604"/>
+  <dimension ref="A1:K605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37318,6 +37344,41 @@
       </c>
       <c r="K604" t="n">
         <v>2.49</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B605" t="n">
+        <v>46.53</v>
+      </c>
+      <c r="C605" t="n">
+        <v>47.83</v>
+      </c>
+      <c r="D605" t="n">
+        <v>46.52</v>
+      </c>
+      <c r="E605" t="n">
+        <v>44.54</v>
+      </c>
+      <c r="F605" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="G605" t="n">
+        <v>46.92</v>
+      </c>
+      <c r="H605" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="I605" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="J605" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="K605" t="n">
+        <v>2.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Otomatik veri güncelleme (07.08.2026 12:29 UTC)
</commit_message>
<xml_diff>
--- a/kredi mevduat/kredi_mevduat.xlsx
+++ b/kredi mevduat/kredi_mevduat.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H605"/>
+  <dimension ref="A1:H606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16168,6 +16168,32 @@
       </c>
       <c r="H605" t="n">
         <v>7.92</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B606" t="n">
+        <v>64.93000000000001</v>
+      </c>
+      <c r="C606" t="n">
+        <v>45.94</v>
+      </c>
+      <c r="D606" t="n">
+        <v>41.84</v>
+      </c>
+      <c r="E606" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="F606" t="n">
+        <v>63.35</v>
+      </c>
+      <c r="G606" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H606" t="n">
+        <v>7.81</v>
       </c>
     </row>
   </sheetData>
@@ -16181,7 +16207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K605"/>
+  <dimension ref="A1:K606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37379,6 +37405,41 @@
       </c>
       <c r="K605" t="n">
         <v>2.58</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B606" t="n">
+        <v>46.25</v>
+      </c>
+      <c r="C606" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="D606" t="n">
+        <v>44.78</v>
+      </c>
+      <c r="E606" t="n">
+        <v>43.12</v>
+      </c>
+      <c r="F606" t="n">
+        <v>38.37</v>
+      </c>
+      <c r="G606" t="n">
+        <v>46.65</v>
+      </c>
+      <c r="H606" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="I606" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="J606" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="K606" t="n">
+        <v>2.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>